<commit_message>
progress: 20 village workbooks (rw-rtx-3070 2026-10-09T02:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Narasingapuram_13.455225_80.128376.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Narasingapuram_13.455225_80.128376.xlsx
@@ -686,6 +686,11 @@
           <t>118</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -693,6 +698,11 @@
           <t>119</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -700,6 +710,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -707,6 +722,11 @@
           <t>120</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -714,6 +734,11 @@
           <t>121</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -721,6 +746,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1A5, 1B, 2A, 2B, 2C, 3A, 3B, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -728,6 +758,11 @@
           <t>123</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5A, 5B, 5C, 5D</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -735,6 +770,11 @@
           <t>124</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3A, 3B, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -742,6 +782,11 @@
           <t>125</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -749,6 +794,11 @@
           <t>126</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -756,6 +806,11 @@
           <t>127</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -763,6 +818,11 @@
           <t>128</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -770,6 +830,11 @@
           <t>129</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -777,6 +842,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -784,6 +854,11 @@
           <t>130</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>-, 1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -791,6 +866,11 @@
           <t>131</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1A, 1B</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -798,6 +878,11 @@
           <t>132</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -805,6 +890,11 @@
           <t>133</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -812,6 +902,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -819,6 +914,11 @@
           <t>135</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -826,6 +926,11 @@
           <t>136</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -833,6 +938,11 @@
           <t>137</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -840,6 +950,11 @@
           <t>138</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -847,6 +962,11 @@
           <t>139</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -854,6 +974,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A1, 3A2, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -861,6 +986,11 @@
           <t>140</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5A1, 5A2, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -868,6 +998,11 @@
           <t>141</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -875,6 +1010,11 @@
           <t>142</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -882,6 +1022,11 @@
           <t>143</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1A1, 2B1A2, 2B1B, 2B2, 2B3</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -889,6 +1034,11 @@
           <t>144</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -896,6 +1046,11 @@
           <t>145</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -903,6 +1058,11 @@
           <t>146</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -910,6 +1070,11 @@
           <t>147</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -917,6 +1082,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -924,6 +1094,11 @@
           <t>149</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -931,6 +1106,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -938,6 +1118,11 @@
           <t>150</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3A, 3B, 4, 5A, 5B1, 5B2, 5C, 5D, 5E, 5F</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -945,6 +1130,11 @@
           <t>151</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1A, 3A1B, 3A1C, 3A1D, 3A2, 3B1A1, 3B1A2, 3B1A3, 3B1A4, 3B1B, 3B1C, 3B1D, 3B1E1, 3B2, 3C, 4</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -952,6 +1142,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3A, 3B, 4A, 4B, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -959,6 +1154,11 @@
           <t>153</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>10, 11, 1A1, 1A2, 1A3, 1A4, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -966,6 +1166,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -973,11 +1178,21 @@
           <t>155</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
           <t>156</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D, 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 20 village workbooks (rw-rtx-3070 2026-10-09T02:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Narasingapuram_13.455225_80.128376.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Narasingapuram_13.455225_80.128376.xlsx
@@ -1202,6 +1202,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1209,6 +1214,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1216,6 +1226,11 @@
           <t>159</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1223,6 +1238,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1230,6 +1250,11 @@
           <t>160</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1237,6 +1262,11 @@
           <t>161</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1244,6 +1274,11 @@
           <t>162</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1251,6 +1286,11 @@
           <t>163</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1258,6 +1298,11 @@
           <t>164</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4A, 4B, 4C, 4D, 4E, 4F</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1265,6 +1310,11 @@
           <t>165</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1272,6 +1322,11 @@
           <t>166</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1279,6 +1334,11 @@
           <t>167</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1286,6 +1346,11 @@
           <t>168</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1293,6 +1358,11 @@
           <t>169</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1300,6 +1370,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1307,6 +1382,11 @@
           <t>170</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 5C, 5D, 5E</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1314,6 +1394,11 @@
           <t>171</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1321,6 +1406,11 @@
           <t>172</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1328,6 +1418,11 @@
           <t>173</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1335,6 +1430,11 @@
           <t>174</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1342,6 +1442,11 @@
           <t>175</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1349,6 +1454,11 @@
           <t>176</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1356,6 +1466,11 @@
           <t>177</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1363,6 +1478,11 @@
           <t>178</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1370,6 +1490,11 @@
           <t>179</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1377,6 +1502,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1384,6 +1514,11 @@
           <t>180</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1391,6 +1526,11 @@
           <t>181</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1398,6 +1538,11 @@
           <t>182</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1405,6 +1550,11 @@
           <t>183</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1412,6 +1562,11 @@
           <t>184</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1419,6 +1574,11 @@
           <t>185</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1426,6 +1586,11 @@
           <t>186</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1433,6 +1598,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1440,6 +1610,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1447,6 +1622,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1454,6 +1634,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1461,6 +1646,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1468,6 +1658,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1475,6 +1670,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1482,6 +1682,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1489,6 +1694,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5A, 5B, 6, 7A, 7B, 7C, 7D, 8A, 8B, 8C, 8D, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1496,6 +1706,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1503,6 +1718,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1510,6 +1730,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1517,6 +1742,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1524,6 +1754,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 3A, 3B, 4, 5, 6A, 6B, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1531,6 +1766,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1538,6 +1778,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 3, 4, 5A, 5B1, 5B2, 6, 7A, 7B, 7C, 7D, 7E, 7F, 7G</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1545,6 +1790,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1552,6 +1802,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2, 2D, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1559,6 +1814,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1566,6 +1826,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1573,6 +1838,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1580,6 +1850,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E1, 3E2, 3F, 3G, 3H, 3I, 3J1, 3J2</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1587,6 +1862,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6A, 6B, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1594,6 +1874,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1601,6 +1886,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1608,6 +1898,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 2, 3, 4A, 4B1A, 4B1B, 4B2, 4B3A, 4B3B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1615,6 +1910,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2A, 2B, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1622,6 +1922,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3A1A1, 3A1B, 3A2, 3A3, 3A4, 3B, 3C, 4, 44, 5A1A1A, 5A2, 5B, 5C, 5D, 5E, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1629,6 +1934,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1636,6 +1946,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1643,6 +1958,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1650,6 +1970,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1657,6 +1982,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1664,6 +1994,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1671,6 +2006,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1678,6 +2018,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1685,6 +2030,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1692,6 +2042,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1699,6 +2054,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1706,6 +2066,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20A, 20B, 21, 22, 23A1, 23A2, 23A3, 23B, 23C1, 23C2, 23C3, 2A, 2B, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1713,6 +2078,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1720,6 +2090,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1727,6 +2102,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1734,6 +2114,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -1741,6 +2126,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C, 11A, 11B, 11C, 1A, 1B, 2, 3, 4, 5A, 5B, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -1748,6 +2138,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 2A, 2B, 2C1, 2C2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -1755,6 +2150,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F1, 2F2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -1762,6 +2162,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D, 1E, 2A, 2B1, 2B2, 3A, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -1769,6 +2174,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -1776,6 +2186,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3, 4, 5A, 5B, 6, 7A, 7B, 7C, 7D, 8</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -1783,11 +2198,21 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
           <t>66</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
         </is>
       </c>
     </row>

</xml_diff>